<commit_message>
Fix email type mss (#190)
* Fix email type mss

* Update AsMailboxMSSProfile.fsh eecdf07f3b23d4f056b2886d9ed92dafae8fc704
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dr-organization.xlsx
+++ b/main/ig/StructureDefinition-as-dr-organization.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AJ$233</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AJ$237</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7538" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7661" uniqueCount="764">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-04T16:55:03+00:00</t>
+    <t>2024-03-05T15:34:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2079,6 +2079,42 @@
   </si>
   <si>
     <t>Organization.telecom:mailbox-mss.extension:emailType</t>
+  </si>
+  <si>
+    <t>Organization.telecom:mailbox-mss.extension:emailType.id</t>
+  </si>
+  <si>
+    <t>Organization.telecom.extension.id</t>
+  </si>
+  <si>
+    <t>Organization.telecom:mailbox-mss.extension:emailType.extension</t>
+  </si>
+  <si>
+    <t>Organization.telecom.extension.extension</t>
+  </si>
+  <si>
+    <t>Organization.telecom:mailbox-mss.extension:emailType.url</t>
+  </si>
+  <si>
+    <t>Organization.telecom.extension.url</t>
+  </si>
+  <si>
+    <t>http://interopsante.org/fhir/StructureDefinition/FrContactPointEmailType</t>
+  </si>
+  <si>
+    <t>Organization.telecom:mailbox-mss.extension:emailType.value[x]</t>
+  </si>
+  <si>
+    <t>Organization.telecom.extension.value[x]</t>
+  </si>
+  <si>
+    <t>&lt;valueCoding xmlns="http://hl7.org/fhir"&gt;
+  &lt;system value="https://mos.esante.gouv.fr/NOS/TRE_R256-TypeMessagerie/FHIR/TRE-R256-TypeMessagerie"/&gt;
+  &lt;code value="MSSANTE"/&gt;
+&lt;/valueCoding&gt;</t>
+  </si>
+  <si>
+    <t>http://interopsante.org/fhir/ValueSet/fr-email-type</t>
   </si>
   <si>
     <t>Organization.telecom:mailbox-mss.extension:as-mailbox-mss-metadata</t>
@@ -2678,7 +2714,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ233"/>
+  <dimension ref="A1:AJ237"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="80.17578125" customWidth="true" bestFit="true"/>
@@ -24119,7 +24155,7 @@
         <v>623</v>
       </c>
       <c r="D210" t="s" s="2">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E210" s="2"/>
       <c r="F210" t="s" s="2">
@@ -24146,9 +24182,7 @@
       <c r="M210" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="N210" t="s" s="2">
-        <v>105</v>
-      </c>
+      <c r="N210" s="2"/>
       <c r="O210" s="2"/>
       <c r="P210" t="s" s="2">
         <v>73</v>
@@ -24217,11 +24251,9 @@
         <v>664</v>
       </c>
       <c r="B211" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="C211" t="s" s="2">
         <v>665</v>
       </c>
+      <c r="C211" s="2"/>
       <c r="D211" t="s" s="2">
         <v>73</v>
       </c>
@@ -24233,7 +24265,7 @@
         <v>81</v>
       </c>
       <c r="H211" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I211" t="s" s="2">
         <v>73</v>
@@ -24242,13 +24274,13 @@
         <v>73</v>
       </c>
       <c r="K211" t="s" s="2">
-        <v>666</v>
+        <v>96</v>
       </c>
       <c r="L211" t="s" s="2">
-        <v>667</v>
+        <v>97</v>
       </c>
       <c r="M211" t="s" s="2">
-        <v>668</v>
+        <v>98</v>
       </c>
       <c r="N211" s="2"/>
       <c r="O211" s="2"/>
@@ -24299,27 +24331,27 @@
         <v>73</v>
       </c>
       <c r="AF211" t="s" s="2">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="AG211" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH211" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI211" t="s" s="2">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="AJ211" t="s" s="2">
-        <v>110</v>
+        <v>73</v>
       </c>
     </row>
     <row r="212" hidden="true">
       <c r="A212" t="s" s="2">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>626</v>
+        <v>667</v>
       </c>
       <c r="C212" s="2"/>
       <c r="D212" t="s" s="2">
@@ -24327,10 +24359,10 @@
       </c>
       <c r="E212" s="2"/>
       <c r="F212" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G212" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="H212" t="s" s="2">
         <v>73</v>
@@ -24339,20 +24371,18 @@
         <v>73</v>
       </c>
       <c r="J212" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K212" t="s" s="2">
-        <v>162</v>
+        <v>102</v>
       </c>
       <c r="L212" t="s" s="2">
-        <v>627</v>
+        <v>479</v>
       </c>
       <c r="M212" t="s" s="2">
-        <v>628</v>
-      </c>
-      <c r="N212" t="s" s="2">
-        <v>379</v>
-      </c>
+        <v>480</v>
+      </c>
+      <c r="N212" s="2"/>
       <c r="O212" s="2"/>
       <c r="P212" t="s" s="2">
         <v>73</v>
@@ -24362,7 +24392,7 @@
         <v>73</v>
       </c>
       <c r="S212" t="s" s="2">
-        <v>670</v>
+        <v>73</v>
       </c>
       <c r="T212" t="s" s="2">
         <v>73</v>
@@ -24377,51 +24407,51 @@
         <v>73</v>
       </c>
       <c r="X212" t="s" s="2">
-        <v>285</v>
+        <v>73</v>
       </c>
       <c r="Y212" t="s" s="2">
-        <v>629</v>
+        <v>73</v>
       </c>
       <c r="Z212" t="s" s="2">
-        <v>630</v>
+        <v>73</v>
       </c>
       <c r="AA212" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AB212" t="s" s="2">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="AC212" t="s" s="2">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AD212" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE212" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="AF212" t="s" s="2">
-        <v>631</v>
+        <v>109</v>
       </c>
       <c r="AG212" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH212" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI212" t="s" s="2">
-        <v>632</v>
+        <v>93</v>
       </c>
       <c r="AJ212" t="s" s="2">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="213" hidden="true">
       <c r="A213" t="s" s="2">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="B213" t="s" s="2">
-        <v>633</v>
+        <v>669</v>
       </c>
       <c r="C213" s="2"/>
       <c r="D213" t="s" s="2">
@@ -24435,35 +24465,33 @@
         <v>81</v>
       </c>
       <c r="H213" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I213" t="s" s="2">
         <v>73</v>
       </c>
       <c r="J213" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K213" t="s" s="2">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="L213" t="s" s="2">
-        <v>672</v>
+        <v>205</v>
       </c>
       <c r="M213" t="s" s="2">
-        <v>635</v>
+        <v>206</v>
       </c>
       <c r="N213" t="s" s="2">
-        <v>636</v>
-      </c>
-      <c r="O213" t="s" s="2">
-        <v>637</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="O213" s="2"/>
       <c r="P213" t="s" s="2">
         <v>73</v>
       </c>
       <c r="Q213" s="2"/>
       <c r="R213" t="s" s="2">
-        <v>73</v>
+        <v>670</v>
       </c>
       <c r="S213" t="s" s="2">
         <v>73</v>
@@ -24505,27 +24533,27 @@
         <v>73</v>
       </c>
       <c r="AF213" t="s" s="2">
-        <v>638</v>
+        <v>209</v>
       </c>
       <c r="AG213" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="AH213" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AI213" t="s" s="2">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="AJ213" t="s" s="2">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="214" hidden="true">
       <c r="A214" t="s" s="2">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B214" t="s" s="2">
-        <v>639</v>
+        <v>672</v>
       </c>
       <c r="C214" s="2"/>
       <c r="D214" t="s" s="2">
@@ -24542,26 +24570,22 @@
         <v>73</v>
       </c>
       <c r="I214" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J214" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K214" t="s" s="2">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="L214" t="s" s="2">
-        <v>640</v>
+        <v>213</v>
       </c>
       <c r="M214" t="s" s="2">
-        <v>641</v>
-      </c>
-      <c r="N214" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="O214" t="s" s="2">
-        <v>643</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="N214" s="2"/>
+      <c r="O214" s="2"/>
       <c r="P214" t="s" s="2">
         <v>73</v>
       </c>
@@ -24570,7 +24594,7 @@
         <v>73</v>
       </c>
       <c r="S214" t="s" s="2">
-        <v>73</v>
+        <v>673</v>
       </c>
       <c r="T214" t="s" s="2">
         <v>73</v>
@@ -24585,13 +24609,11 @@
         <v>73</v>
       </c>
       <c r="X214" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="Y214" t="s" s="2">
-        <v>644</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="Y214" s="2"/>
       <c r="Z214" t="s" s="2">
-        <v>645</v>
+        <v>674</v>
       </c>
       <c r="AA214" t="s" s="2">
         <v>73</v>
@@ -24609,7 +24631,7 @@
         <v>73</v>
       </c>
       <c r="AF214" t="s" s="2">
-        <v>646</v>
+        <v>215</v>
       </c>
       <c r="AG214" t="s" s="2">
         <v>74</v>
@@ -24629,9 +24651,11 @@
         <v>675</v>
       </c>
       <c r="B215" t="s" s="2">
-        <v>647</v>
-      </c>
-      <c r="C215" s="2"/>
+        <v>621</v>
+      </c>
+      <c r="C215" t="s" s="2">
+        <v>676</v>
+      </c>
       <c r="D215" t="s" s="2">
         <v>73</v>
       </c>
@@ -24643,26 +24667,24 @@
         <v>81</v>
       </c>
       <c r="H215" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="I215" t="s" s="2">
         <v>73</v>
       </c>
       <c r="J215" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K215" t="s" s="2">
-        <v>648</v>
+        <v>677</v>
       </c>
       <c r="L215" t="s" s="2">
-        <v>649</v>
+        <v>678</v>
       </c>
       <c r="M215" t="s" s="2">
-        <v>650</v>
-      </c>
-      <c r="N215" t="s" s="2">
-        <v>651</v>
-      </c>
+        <v>679</v>
+      </c>
+      <c r="N215" s="2"/>
       <c r="O215" s="2"/>
       <c r="P215" t="s" s="2">
         <v>73</v>
@@ -24711,27 +24733,27 @@
         <v>73</v>
       </c>
       <c r="AF215" t="s" s="2">
-        <v>652</v>
+        <v>109</v>
       </c>
       <c r="AG215" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH215" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI215" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ215" t="s" s="2">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="216" hidden="true">
       <c r="A216" t="s" s="2">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B216" t="s" s="2">
-        <v>653</v>
+        <v>626</v>
       </c>
       <c r="C216" s="2"/>
       <c r="D216" t="s" s="2">
@@ -24739,7 +24761,7 @@
       </c>
       <c r="E216" s="2"/>
       <c r="F216" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G216" t="s" s="2">
         <v>81</v>
@@ -24754,16 +24776,16 @@
         <v>82</v>
       </c>
       <c r="K216" t="s" s="2">
-        <v>212</v>
+        <v>162</v>
       </c>
       <c r="L216" t="s" s="2">
-        <v>654</v>
+        <v>627</v>
       </c>
       <c r="M216" t="s" s="2">
-        <v>655</v>
+        <v>628</v>
       </c>
       <c r="N216" t="s" s="2">
-        <v>314</v>
+        <v>379</v>
       </c>
       <c r="O216" s="2"/>
       <c r="P216" t="s" s="2">
@@ -24774,7 +24796,7 @@
         <v>73</v>
       </c>
       <c r="S216" t="s" s="2">
-        <v>73</v>
+        <v>681</v>
       </c>
       <c r="T216" t="s" s="2">
         <v>73</v>
@@ -24789,13 +24811,13 @@
         <v>73</v>
       </c>
       <c r="X216" t="s" s="2">
-        <v>73</v>
+        <v>285</v>
       </c>
       <c r="Y216" t="s" s="2">
-        <v>73</v>
+        <v>629</v>
       </c>
       <c r="Z216" t="s" s="2">
-        <v>73</v>
+        <v>630</v>
       </c>
       <c r="AA216" t="s" s="2">
         <v>73</v>
@@ -24813,7 +24835,7 @@
         <v>73</v>
       </c>
       <c r="AF216" t="s" s="2">
-        <v>656</v>
+        <v>631</v>
       </c>
       <c r="AG216" t="s" s="2">
         <v>74</v>
@@ -24822,18 +24844,18 @@
         <v>81</v>
       </c>
       <c r="AI216" t="s" s="2">
-        <v>93</v>
+        <v>632</v>
       </c>
       <c r="AJ216" t="s" s="2">
-        <v>316</v>
+        <v>94</v>
       </c>
     </row>
     <row r="217" hidden="true">
       <c r="A217" t="s" s="2">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="B217" t="s" s="2">
-        <v>677</v>
+        <v>633</v>
       </c>
       <c r="C217" s="2"/>
       <c r="D217" t="s" s="2">
@@ -24841,10 +24863,10 @@
       </c>
       <c r="E217" s="2"/>
       <c r="F217" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G217" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H217" t="s" s="2">
         <v>82</v>
@@ -24853,22 +24875,22 @@
         <v>73</v>
       </c>
       <c r="J217" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K217" t="s" s="2">
-        <v>678</v>
+        <v>96</v>
       </c>
       <c r="L217" t="s" s="2">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="M217" t="s" s="2">
-        <v>680</v>
+        <v>635</v>
       </c>
       <c r="N217" t="s" s="2">
-        <v>681</v>
+        <v>636</v>
       </c>
       <c r="O217" t="s" s="2">
-        <v>682</v>
+        <v>637</v>
       </c>
       <c r="P217" t="s" s="2">
         <v>73</v>
@@ -24917,19 +24939,19 @@
         <v>73</v>
       </c>
       <c r="AF217" t="s" s="2">
-        <v>677</v>
+        <v>638</v>
       </c>
       <c r="AG217" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH217" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI217" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ217" t="s" s="2">
-        <v>683</v>
+        <v>94</v>
       </c>
     </row>
     <row r="218" hidden="true">
@@ -24937,7 +24959,7 @@
         <v>684</v>
       </c>
       <c r="B218" t="s" s="2">
-        <v>684</v>
+        <v>639</v>
       </c>
       <c r="C218" s="2"/>
       <c r="D218" t="s" s="2">
@@ -24954,25 +24976,25 @@
         <v>73</v>
       </c>
       <c r="I218" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J218" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K218" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="L218" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="M218" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="N218" t="s" s="2">
         <v>685</v>
       </c>
-      <c r="L218" t="s" s="2">
-        <v>686</v>
-      </c>
-      <c r="M218" t="s" s="2">
-        <v>687</v>
-      </c>
-      <c r="N218" t="s" s="2">
-        <v>688</v>
-      </c>
       <c r="O218" t="s" s="2">
-        <v>689</v>
+        <v>643</v>
       </c>
       <c r="P218" t="s" s="2">
         <v>73</v>
@@ -24997,13 +25019,13 @@
         <v>73</v>
       </c>
       <c r="X218" t="s" s="2">
-        <v>73</v>
+        <v>285</v>
       </c>
       <c r="Y218" t="s" s="2">
-        <v>73</v>
+        <v>644</v>
       </c>
       <c r="Z218" t="s" s="2">
-        <v>73</v>
+        <v>645</v>
       </c>
       <c r="AA218" t="s" s="2">
         <v>73</v>
@@ -25021,7 +25043,7 @@
         <v>73</v>
       </c>
       <c r="AF218" t="s" s="2">
-        <v>684</v>
+        <v>646</v>
       </c>
       <c r="AG218" t="s" s="2">
         <v>74</v>
@@ -25033,15 +25055,15 @@
         <v>93</v>
       </c>
       <c r="AJ218" t="s" s="2">
-        <v>323</v>
+        <v>94</v>
       </c>
     </row>
     <row r="219" hidden="true">
       <c r="A219" t="s" s="2">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="B219" t="s" s="2">
-        <v>690</v>
+        <v>647</v>
       </c>
       <c r="C219" s="2"/>
       <c r="D219" t="s" s="2">
@@ -25061,18 +25083,20 @@
         <v>73</v>
       </c>
       <c r="J219" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K219" t="s" s="2">
-        <v>96</v>
+        <v>648</v>
       </c>
       <c r="L219" t="s" s="2">
-        <v>97</v>
+        <v>649</v>
       </c>
       <c r="M219" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="N219" s="2"/>
+        <v>650</v>
+      </c>
+      <c r="N219" t="s" s="2">
+        <v>651</v>
+      </c>
       <c r="O219" s="2"/>
       <c r="P219" t="s" s="2">
         <v>73</v>
@@ -25121,7 +25145,7 @@
         <v>73</v>
       </c>
       <c r="AF219" t="s" s="2">
-        <v>99</v>
+        <v>652</v>
       </c>
       <c r="AG219" t="s" s="2">
         <v>74</v>
@@ -25130,29 +25154,29 @@
         <v>81</v>
       </c>
       <c r="AI219" t="s" s="2">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="AJ219" t="s" s="2">
-        <v>73</v>
+        <v>94</v>
       </c>
     </row>
     <row r="220" hidden="true">
       <c r="A220" t="s" s="2">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="B220" t="s" s="2">
-        <v>691</v>
+        <v>653</v>
       </c>
       <c r="C220" s="2"/>
       <c r="D220" t="s" s="2">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E220" s="2"/>
       <c r="F220" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G220" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H220" t="s" s="2">
         <v>73</v>
@@ -25161,19 +25185,19 @@
         <v>73</v>
       </c>
       <c r="J220" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K220" t="s" s="2">
-        <v>102</v>
+        <v>212</v>
       </c>
       <c r="L220" t="s" s="2">
-        <v>103</v>
+        <v>654</v>
       </c>
       <c r="M220" t="s" s="2">
-        <v>104</v>
+        <v>655</v>
       </c>
       <c r="N220" t="s" s="2">
-        <v>105</v>
+        <v>314</v>
       </c>
       <c r="O220" s="2"/>
       <c r="P220" t="s" s="2">
@@ -25211,39 +25235,39 @@
         <v>73</v>
       </c>
       <c r="AB220" t="s" s="2">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="AC220" t="s" s="2">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="AD220" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE220" t="s" s="2">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="AF220" t="s" s="2">
-        <v>109</v>
+        <v>656</v>
       </c>
       <c r="AG220" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH220" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI220" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ220" t="s" s="2">
-        <v>110</v>
+        <v>316</v>
       </c>
     </row>
     <row r="221" hidden="true">
       <c r="A221" t="s" s="2">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="B221" t="s" s="2">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="C221" s="2"/>
       <c r="D221" t="s" s="2">
@@ -25254,30 +25278,32 @@
         <v>74</v>
       </c>
       <c r="G221" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H221" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="I221" t="s" s="2">
         <v>73</v>
       </c>
       <c r="J221" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K221" t="s" s="2">
-        <v>96</v>
+        <v>689</v>
       </c>
       <c r="L221" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="M221" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="N221" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="O221" t="s" s="2">
         <v>693</v>
       </c>
-      <c r="M221" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="N221" t="s" s="2">
-        <v>695</v>
-      </c>
-      <c r="O221" s="2"/>
       <c r="P221" t="s" s="2">
         <v>73</v>
       </c>
@@ -25325,27 +25351,27 @@
         <v>73</v>
       </c>
       <c r="AF221" t="s" s="2">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="AG221" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH221" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI221" t="s" s="2">
-        <v>697</v>
+        <v>93</v>
       </c>
       <c r="AJ221" t="s" s="2">
-        <v>94</v>
+        <v>694</v>
       </c>
     </row>
     <row r="222" hidden="true">
       <c r="A222" t="s" s="2">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="B222" t="s" s="2">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="C222" s="2"/>
       <c r="D222" t="s" s="2">
@@ -25368,18 +25394,20 @@
         <v>82</v>
       </c>
       <c r="K222" t="s" s="2">
-        <v>128</v>
+        <v>696</v>
       </c>
       <c r="L222" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="M222" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="N222" t="s" s="2">
         <v>699</v>
       </c>
-      <c r="M222" t="s" s="2">
+      <c r="O222" t="s" s="2">
         <v>700</v>
       </c>
-      <c r="N222" t="s" s="2">
-        <v>701</v>
-      </c>
-      <c r="O222" s="2"/>
       <c r="P222" t="s" s="2">
         <v>73</v>
       </c>
@@ -25403,13 +25431,13 @@
         <v>73</v>
       </c>
       <c r="X222" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
       <c r="Y222" t="s" s="2">
-        <v>702</v>
+        <v>73</v>
       </c>
       <c r="Z222" t="s" s="2">
-        <v>474</v>
+        <v>73</v>
       </c>
       <c r="AA222" t="s" s="2">
         <v>73</v>
@@ -25427,7 +25455,7 @@
         <v>73</v>
       </c>
       <c r="AF222" t="s" s="2">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="AG222" t="s" s="2">
         <v>74</v>
@@ -25439,15 +25467,15 @@
         <v>93</v>
       </c>
       <c r="AJ222" t="s" s="2">
-        <v>94</v>
+        <v>323</v>
       </c>
     </row>
     <row r="223" hidden="true">
       <c r="A223" t="s" s="2">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="B223" t="s" s="2">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C223" s="2"/>
       <c r="D223" t="s" s="2">
@@ -25467,20 +25495,18 @@
         <v>73</v>
       </c>
       <c r="J223" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K223" t="s" s="2">
-        <v>271</v>
+        <v>96</v>
       </c>
       <c r="L223" t="s" s="2">
-        <v>705</v>
+        <v>97</v>
       </c>
       <c r="M223" t="s" s="2">
-        <v>706</v>
-      </c>
-      <c r="N223" t="s" s="2">
-        <v>707</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="N223" s="2"/>
       <c r="O223" s="2"/>
       <c r="P223" t="s" s="2">
         <v>73</v>
@@ -25529,7 +25555,7 @@
         <v>73</v>
       </c>
       <c r="AF223" t="s" s="2">
-        <v>708</v>
+        <v>99</v>
       </c>
       <c r="AG223" t="s" s="2">
         <v>74</v>
@@ -25538,29 +25564,29 @@
         <v>81</v>
       </c>
       <c r="AI223" t="s" s="2">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="AJ223" t="s" s="2">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="224" hidden="true">
       <c r="A224" t="s" s="2">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="B224" t="s" s="2">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="C224" s="2"/>
       <c r="D224" t="s" s="2">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="E224" s="2"/>
       <c r="F224" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G224" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H224" t="s" s="2">
         <v>73</v>
@@ -25569,19 +25595,19 @@
         <v>73</v>
       </c>
       <c r="J224" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K224" t="s" s="2">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="L224" t="s" s="2">
-        <v>710</v>
+        <v>103</v>
       </c>
       <c r="M224" t="s" s="2">
-        <v>711</v>
+        <v>104</v>
       </c>
       <c r="N224" t="s" s="2">
-        <v>712</v>
+        <v>105</v>
       </c>
       <c r="O224" s="2"/>
       <c r="P224" t="s" s="2">
@@ -25619,39 +25645,39 @@
         <v>73</v>
       </c>
       <c r="AB224" t="s" s="2">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="AC224" t="s" s="2">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AD224" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE224" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="AF224" t="s" s="2">
-        <v>713</v>
+        <v>109</v>
       </c>
       <c r="AG224" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH224" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI224" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ224" t="s" s="2">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="225" hidden="true">
       <c r="A225" t="s" s="2">
-        <v>714</v>
+        <v>703</v>
       </c>
       <c r="B225" t="s" s="2">
-        <v>714</v>
+        <v>703</v>
       </c>
       <c r="C225" s="2"/>
       <c r="D225" t="s" s="2">
@@ -25662,7 +25688,7 @@
         <v>74</v>
       </c>
       <c r="G225" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H225" t="s" s="2">
         <v>73</v>
@@ -25671,23 +25697,21 @@
         <v>73</v>
       </c>
       <c r="J225" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K225" t="s" s="2">
-        <v>715</v>
+        <v>96</v>
       </c>
       <c r="L225" t="s" s="2">
-        <v>716</v>
+        <v>704</v>
       </c>
       <c r="M225" t="s" s="2">
-        <v>717</v>
+        <v>705</v>
       </c>
       <c r="N225" t="s" s="2">
-        <v>718</v>
-      </c>
-      <c r="O225" t="s" s="2">
-        <v>719</v>
-      </c>
+        <v>706</v>
+      </c>
+      <c r="O225" s="2"/>
       <c r="P225" t="s" s="2">
         <v>73</v>
       </c>
@@ -25735,16 +25759,16 @@
         <v>73</v>
       </c>
       <c r="AF225" t="s" s="2">
-        <v>714</v>
+        <v>707</v>
       </c>
       <c r="AG225" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH225" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI225" t="s" s="2">
-        <v>93</v>
+        <v>708</v>
       </c>
       <c r="AJ225" t="s" s="2">
         <v>94</v>
@@ -25752,10 +25776,10 @@
     </row>
     <row r="226" hidden="true">
       <c r="A226" t="s" s="2">
-        <v>720</v>
+        <v>709</v>
       </c>
       <c r="B226" t="s" s="2">
-        <v>720</v>
+        <v>709</v>
       </c>
       <c r="C226" s="2"/>
       <c r="D226" t="s" s="2">
@@ -25775,18 +25799,20 @@
         <v>73</v>
       </c>
       <c r="J226" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K226" t="s" s="2">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="L226" t="s" s="2">
-        <v>97</v>
+        <v>710</v>
       </c>
       <c r="M226" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="N226" s="2"/>
+        <v>711</v>
+      </c>
+      <c r="N226" t="s" s="2">
+        <v>712</v>
+      </c>
       <c r="O226" s="2"/>
       <c r="P226" t="s" s="2">
         <v>73</v>
@@ -25811,13 +25837,13 @@
         <v>73</v>
       </c>
       <c r="X226" t="s" s="2">
-        <v>73</v>
+        <v>144</v>
       </c>
       <c r="Y226" t="s" s="2">
-        <v>73</v>
+        <v>713</v>
       </c>
       <c r="Z226" t="s" s="2">
-        <v>73</v>
+        <v>474</v>
       </c>
       <c r="AA226" t="s" s="2">
         <v>73</v>
@@ -25835,7 +25861,7 @@
         <v>73</v>
       </c>
       <c r="AF226" t="s" s="2">
-        <v>99</v>
+        <v>714</v>
       </c>
       <c r="AG226" t="s" s="2">
         <v>74</v>
@@ -25844,29 +25870,29 @@
         <v>81</v>
       </c>
       <c r="AI226" t="s" s="2">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="AJ226" t="s" s="2">
-        <v>73</v>
+        <v>94</v>
       </c>
     </row>
     <row r="227" hidden="true">
       <c r="A227" t="s" s="2">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="B227" t="s" s="2">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="C227" s="2"/>
       <c r="D227" t="s" s="2">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E227" s="2"/>
       <c r="F227" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G227" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H227" t="s" s="2">
         <v>73</v>
@@ -25875,19 +25901,19 @@
         <v>73</v>
       </c>
       <c r="J227" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K227" t="s" s="2">
-        <v>102</v>
+        <v>271</v>
       </c>
       <c r="L227" t="s" s="2">
-        <v>103</v>
+        <v>716</v>
       </c>
       <c r="M227" t="s" s="2">
-        <v>104</v>
+        <v>717</v>
       </c>
       <c r="N227" t="s" s="2">
-        <v>105</v>
+        <v>718</v>
       </c>
       <c r="O227" s="2"/>
       <c r="P227" t="s" s="2">
@@ -25925,75 +25951,73 @@
         <v>73</v>
       </c>
       <c r="AB227" t="s" s="2">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="AC227" t="s" s="2">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="AD227" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE227" t="s" s="2">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="AF227" t="s" s="2">
-        <v>109</v>
+        <v>719</v>
       </c>
       <c r="AG227" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH227" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI227" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ227" t="s" s="2">
-        <v>110</v>
+        <v>94</v>
       </c>
     </row>
     <row r="228" hidden="true">
       <c r="A228" t="s" s="2">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B228" t="s" s="2">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="C228" s="2"/>
       <c r="D228" t="s" s="2">
-        <v>723</v>
+        <v>73</v>
       </c>
       <c r="E228" s="2"/>
       <c r="F228" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G228" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H228" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I228" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J228" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K228" t="s" s="2">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="L228" t="s" s="2">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="M228" t="s" s="2">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="N228" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="O228" t="s" s="2">
-        <v>268</v>
-      </c>
+        <v>723</v>
+      </c>
+      <c r="O228" s="2"/>
       <c r="P228" t="s" s="2">
         <v>73</v>
       </c>
@@ -26041,27 +26065,27 @@
         <v>73</v>
       </c>
       <c r="AF228" t="s" s="2">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="AG228" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH228" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI228" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ228" t="s" s="2">
-        <v>110</v>
+        <v>94</v>
       </c>
     </row>
     <row r="229" hidden="true">
       <c r="A229" t="s" s="2">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="B229" t="s" s="2">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C229" s="2"/>
       <c r="D229" t="s" s="2">
@@ -26072,7 +26096,7 @@
         <v>74</v>
       </c>
       <c r="G229" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H229" t="s" s="2">
         <v>73</v>
@@ -26084,19 +26108,19 @@
         <v>73</v>
       </c>
       <c r="K229" t="s" s="2">
-        <v>290</v>
+        <v>726</v>
       </c>
       <c r="L229" t="s" s="2">
+        <v>727</v>
+      </c>
+      <c r="M229" t="s" s="2">
         <v>728</v>
       </c>
-      <c r="M229" t="s" s="2">
+      <c r="N229" t="s" s="2">
         <v>729</v>
       </c>
-      <c r="N229" t="s" s="2">
+      <c r="O229" t="s" s="2">
         <v>730</v>
-      </c>
-      <c r="O229" t="s" s="2">
-        <v>731</v>
       </c>
       <c r="P229" t="s" s="2">
         <v>73</v>
@@ -26121,13 +26145,13 @@
         <v>73</v>
       </c>
       <c r="X229" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
       <c r="Y229" t="s" s="2">
-        <v>732</v>
+        <v>73</v>
       </c>
       <c r="Z229" t="s" s="2">
-        <v>733</v>
+        <v>73</v>
       </c>
       <c r="AA229" t="s" s="2">
         <v>73</v>
@@ -26145,13 +26169,13 @@
         <v>73</v>
       </c>
       <c r="AF229" t="s" s="2">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="AG229" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH229" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI229" t="s" s="2">
         <v>93</v>
@@ -26162,10 +26186,10 @@
     </row>
     <row r="230" hidden="true">
       <c r="A230" t="s" s="2">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="B230" t="s" s="2">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="C230" s="2"/>
       <c r="D230" t="s" s="2">
@@ -26188,20 +26212,16 @@
         <v>73</v>
       </c>
       <c r="K230" t="s" s="2">
-        <v>735</v>
+        <v>96</v>
       </c>
       <c r="L230" t="s" s="2">
-        <v>736</v>
+        <v>97</v>
       </c>
       <c r="M230" t="s" s="2">
-        <v>737</v>
-      </c>
-      <c r="N230" t="s" s="2">
-        <v>738</v>
-      </c>
-      <c r="O230" t="s" s="2">
-        <v>739</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="N230" s="2"/>
+      <c r="O230" s="2"/>
       <c r="P230" t="s" s="2">
         <v>73</v>
       </c>
@@ -26249,7 +26269,7 @@
         <v>73</v>
       </c>
       <c r="AF230" t="s" s="2">
-        <v>734</v>
+        <v>99</v>
       </c>
       <c r="AG230" t="s" s="2">
         <v>74</v>
@@ -26258,22 +26278,22 @@
         <v>81</v>
       </c>
       <c r="AI230" t="s" s="2">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="AJ230" t="s" s="2">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="231" hidden="true">
       <c r="A231" t="s" s="2">
-        <v>740</v>
+        <v>732</v>
       </c>
       <c r="B231" t="s" s="2">
-        <v>740</v>
+        <v>732</v>
       </c>
       <c r="C231" s="2"/>
       <c r="D231" t="s" s="2">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="E231" s="2"/>
       <c r="F231" t="s" s="2">
@@ -26292,18 +26312,18 @@
         <v>73</v>
       </c>
       <c r="K231" t="s" s="2">
-        <v>612</v>
+        <v>102</v>
       </c>
       <c r="L231" t="s" s="2">
-        <v>741</v>
+        <v>103</v>
       </c>
       <c r="M231" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="N231" s="2"/>
-      <c r="O231" t="s" s="2">
-        <v>742</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N231" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="O231" s="2"/>
       <c r="P231" t="s" s="2">
         <v>73</v>
       </c>
@@ -26339,19 +26359,19 @@
         <v>73</v>
       </c>
       <c r="AB231" t="s" s="2">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="AC231" t="s" s="2">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AD231" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE231" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="AF231" t="s" s="2">
-        <v>740</v>
+        <v>109</v>
       </c>
       <c r="AG231" t="s" s="2">
         <v>74</v>
@@ -26363,50 +26383,50 @@
         <v>93</v>
       </c>
       <c r="AJ231" t="s" s="2">
-        <v>743</v>
+        <v>110</v>
       </c>
     </row>
     <row r="232" hidden="true">
       <c r="A232" t="s" s="2">
-        <v>744</v>
+        <v>733</v>
       </c>
       <c r="B232" t="s" s="2">
-        <v>744</v>
+        <v>733</v>
       </c>
       <c r="C232" s="2"/>
       <c r="D232" t="s" s="2">
-        <v>73</v>
+        <v>734</v>
       </c>
       <c r="E232" s="2"/>
       <c r="F232" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G232" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H232" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I232" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J232" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K232" t="s" s="2">
-        <v>745</v>
+        <v>102</v>
       </c>
       <c r="L232" t="s" s="2">
-        <v>746</v>
+        <v>735</v>
       </c>
       <c r="M232" t="s" s="2">
-        <v>680</v>
+        <v>736</v>
       </c>
       <c r="N232" t="s" s="2">
-        <v>681</v>
+        <v>105</v>
       </c>
       <c r="O232" t="s" s="2">
-        <v>747</v>
+        <v>268</v>
       </c>
       <c r="P232" t="s" s="2">
         <v>73</v>
@@ -26455,27 +26475,27 @@
         <v>73</v>
       </c>
       <c r="AF232" t="s" s="2">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="AG232" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH232" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI232" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ232" t="s" s="2">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="233" hidden="true">
       <c r="A233" t="s" s="2">
-        <v>748</v>
+        <v>738</v>
       </c>
       <c r="B233" t="s" s="2">
-        <v>748</v>
+        <v>738</v>
       </c>
       <c r="C233" s="2"/>
       <c r="D233" t="s" s="2">
@@ -26486,10 +26506,10 @@
         <v>74</v>
       </c>
       <c r="G233" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H233" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I233" t="s" s="2">
         <v>73</v>
@@ -26498,19 +26518,19 @@
         <v>73</v>
       </c>
       <c r="K233" t="s" s="2">
-        <v>749</v>
+        <v>290</v>
       </c>
       <c r="L233" t="s" s="2">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="M233" t="s" s="2">
-        <v>751</v>
+        <v>740</v>
       </c>
       <c r="N233" t="s" s="2">
-        <v>688</v>
+        <v>741</v>
       </c>
       <c r="O233" t="s" s="2">
-        <v>752</v>
+        <v>742</v>
       </c>
       <c r="P233" t="s" s="2">
         <v>73</v>
@@ -26535,13 +26555,13 @@
         <v>73</v>
       </c>
       <c r="X233" t="s" s="2">
-        <v>73</v>
+        <v>144</v>
       </c>
       <c r="Y233" t="s" s="2">
-        <v>73</v>
+        <v>743</v>
       </c>
       <c r="Z233" t="s" s="2">
-        <v>73</v>
+        <v>744</v>
       </c>
       <c r="AA233" t="s" s="2">
         <v>73</v>
@@ -26559,23 +26579,437 @@
         <v>73</v>
       </c>
       <c r="AF233" t="s" s="2">
-        <v>748</v>
+        <v>738</v>
       </c>
       <c r="AG233" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH233" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI233" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ233" t="s" s="2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="234" hidden="true">
+      <c r="A234" t="s" s="2">
+        <v>745</v>
+      </c>
+      <c r="B234" t="s" s="2">
+        <v>745</v>
+      </c>
+      <c r="C234" s="2"/>
+      <c r="D234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E234" s="2"/>
+      <c r="F234" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G234" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K234" t="s" s="2">
+        <v>746</v>
+      </c>
+      <c r="L234" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="M234" t="s" s="2">
+        <v>748</v>
+      </c>
+      <c r="N234" t="s" s="2">
+        <v>749</v>
+      </c>
+      <c r="O234" t="s" s="2">
+        <v>750</v>
+      </c>
+      <c r="P234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q234" s="2"/>
+      <c r="R234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE234" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF234" t="s" s="2">
+        <v>745</v>
+      </c>
+      <c r="AG234" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH234" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI234" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ234" t="s" s="2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="235" hidden="true">
+      <c r="A235" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="B235" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="C235" s="2"/>
+      <c r="D235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E235" s="2"/>
+      <c r="F235" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G235" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K235" t="s" s="2">
+        <v>612</v>
+      </c>
+      <c r="L235" t="s" s="2">
+        <v>752</v>
+      </c>
+      <c r="M235" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="N235" s="2"/>
+      <c r="O235" t="s" s="2">
+        <v>753</v>
+      </c>
+      <c r="P235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q235" s="2"/>
+      <c r="R235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE235" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF235" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="AG235" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH235" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI235" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ235" t="s" s="2">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="236" hidden="true">
+      <c r="A236" t="s" s="2">
+        <v>755</v>
+      </c>
+      <c r="B236" t="s" s="2">
+        <v>755</v>
+      </c>
+      <c r="C236" s="2"/>
+      <c r="D236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E236" s="2"/>
+      <c r="F236" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G236" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K236" t="s" s="2">
+        <v>756</v>
+      </c>
+      <c r="L236" t="s" s="2">
+        <v>757</v>
+      </c>
+      <c r="M236" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="N236" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="O236" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="P236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q236" s="2"/>
+      <c r="R236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE236" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF236" t="s" s="2">
+        <v>755</v>
+      </c>
+      <c r="AG236" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH236" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI236" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ236" t="s" s="2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="237" hidden="true">
+      <c r="A237" t="s" s="2">
+        <v>759</v>
+      </c>
+      <c r="B237" t="s" s="2">
+        <v>759</v>
+      </c>
+      <c r="C237" s="2"/>
+      <c r="D237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E237" s="2"/>
+      <c r="F237" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G237" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H237" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K237" t="s" s="2">
+        <v>760</v>
+      </c>
+      <c r="L237" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="M237" t="s" s="2">
+        <v>762</v>
+      </c>
+      <c r="N237" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="O237" t="s" s="2">
+        <v>763</v>
+      </c>
+      <c r="P237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q237" s="2"/>
+      <c r="R237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE237" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF237" t="s" s="2">
+        <v>759</v>
+      </c>
+      <c r="AG237" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH237" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI237" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ237" t="s" s="2">
         <v>323</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ233">
+  <autoFilter ref="A1:AJ237">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -26585,7 +27019,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI232">
+  <conditionalFormatting sqref="A2:AI236">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>